<commit_message>
Learning about feature engineering
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Belajar\udemy\Data analyst Bootcamp\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8DEF6B-8179-4580-B8D3-9B623C3387AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6B6417-3BBD-49A6-9B1E-1DD2E7140D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C0FCC827-97E3-4E98-9870-BE76B2B14A0C}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>jam</t>
   </si>
@@ -73,6 +73,12 @@
   </si>
   <si>
     <t>jumlah materi selesai</t>
+  </si>
+  <si>
+    <t>burnt out</t>
+  </si>
+  <si>
+    <t>family gathering satangair</t>
   </si>
 </sst>
 </file>
@@ -91,12 +97,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -111,10 +123,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -433,7 +447,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.33203125" customWidth="1"/>
+    <col min="6" max="6" width="21.88671875" customWidth="1"/>
     <col min="7" max="8" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -915,28 +929,83 @@
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B24">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3">
         <v>23</v>
       </c>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="4">
+        <v>45891</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>7</v>
+      </c>
       <c r="B25">
         <v>24</v>
       </c>
+      <c r="C25" s="1">
+        <f>F25/$G$2*100</f>
+        <v>32.372505543237253</v>
+      </c>
+      <c r="D25">
+        <f>AVERAGE(A20:A25)</f>
+        <v>6.9</v>
+      </c>
+      <c r="E25" s="2">
+        <v>45892</v>
+      </c>
+      <c r="F25">
+        <v>146</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B26">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3">
         <v>25</v>
       </c>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="4">
+        <v>45893</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2</v>
+      </c>
       <c r="B27">
         <v>26</v>
+      </c>
+      <c r="C27" s="1">
+        <f>F27/$G$2*100</f>
+        <v>32.8159645232816</v>
+      </c>
+      <c r="D27">
+        <f>AVERAGE(A22:A27)</f>
+        <v>5.75</v>
+      </c>
+      <c r="E27" s="2">
+        <v>45894</v>
+      </c>
+      <c r="F27">
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="B28">
         <v>27</v>
+      </c>
+      <c r="E28" s="2">
+        <v>45895</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Learning About Exploratory Data Analysis and Feature Engineering
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Belajar\udemy\Data analyst Bootcamp\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA6B6417-3BBD-49A6-9B1E-1DD2E7140D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11AB64F4-5956-4504-8DAD-3A8459ADCA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C0FCC827-97E3-4E98-9870-BE76B2B14A0C}"/>
   </bookViews>
@@ -1001,11 +1001,25 @@
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>6.25</v>
+      </c>
       <c r="B28">
         <v>27</v>
       </c>
+      <c r="C28" s="1">
+        <f>F28/$G$2*100</f>
+        <v>33.924611973392459</v>
+      </c>
+      <c r="D28">
+        <f>AVERAGE(A23:A28)</f>
+        <v>5.3125</v>
+      </c>
       <c r="E28" s="2">
         <v>45895</v>
+      </c>
+      <c r="F28" s="3">
+        <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Learning about Linear Regression, Ridge, Lasso, and ElasticNet ML Algorithm
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Belajar\udemy\Data analyst Bootcamp\python\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11AB64F4-5956-4504-8DAD-3A8459ADCA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDE3CAEF-3323-400A-82CE-B0A548874CDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C0FCC827-97E3-4E98-9870-BE76B2B14A0C}"/>
   </bookViews>
@@ -123,12 +123,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,6 +450,7 @@
     <col min="5" max="5" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="21.88671875" customWidth="1"/>
     <col min="7" max="8" width="10.5546875" customWidth="1"/>
+    <col min="10" max="10" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
@@ -986,17 +988,17 @@
         <v>26</v>
       </c>
       <c r="C27" s="1">
-        <f>F27/$G$2*100</f>
+        <f t="shared" ref="C27:C33" si="1">F27/$G$2*100</f>
         <v>32.8159645232816</v>
       </c>
       <c r="D27">
-        <f>AVERAGE(A22:A27)</f>
+        <f t="shared" ref="D27:D32" si="2">AVERAGE(A22:A27)</f>
         <v>5.75</v>
       </c>
       <c r="E27" s="2">
         <v>45894</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="5">
         <v>148</v>
       </c>
     </row>
@@ -1008,116 +1010,201 @@
         <v>27</v>
       </c>
       <c r="C28" s="1">
-        <f>F28/$G$2*100</f>
+        <f t="shared" si="1"/>
         <v>33.924611973392459</v>
       </c>
       <c r="D28">
-        <f>AVERAGE(A23:A28)</f>
+        <f t="shared" si="2"/>
         <v>5.3125</v>
       </c>
       <c r="E28" s="2">
         <v>45895</v>
       </c>
-      <c r="F28" s="3">
+      <c r="F28" s="5">
         <v>153</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>10</v>
+      </c>
       <c r="B29">
         <v>28</v>
       </c>
+      <c r="C29" s="1">
+        <f t="shared" si="1"/>
+        <v>34.811529933481154</v>
+      </c>
+      <c r="D29">
+        <f t="shared" si="2"/>
+        <v>6.3125</v>
+      </c>
+      <c r="E29" s="2">
+        <v>45896</v>
+      </c>
+      <c r="F29" s="5">
+        <v>157</v>
+      </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>8.5</v>
+      </c>
       <c r="B30">
         <v>29</v>
       </c>
+      <c r="C30" s="1">
+        <f t="shared" si="1"/>
+        <v>37.250554323725055</v>
+      </c>
+      <c r="D30">
+        <f t="shared" si="2"/>
+        <v>6.75</v>
+      </c>
+      <c r="E30" s="2">
+        <v>45897</v>
+      </c>
+      <c r="F30" s="5">
+        <v>168</v>
+      </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>7</v>
+      </c>
       <c r="B31">
         <v>30</v>
       </c>
+      <c r="C31" s="1">
+        <f t="shared" si="1"/>
+        <v>38.137472283813743</v>
+      </c>
+      <c r="D31">
+        <f t="shared" si="2"/>
+        <v>6.75</v>
+      </c>
+      <c r="E31" s="2">
+        <v>45898</v>
+      </c>
+      <c r="F31" s="5">
+        <v>172</v>
+      </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>2.6</v>
+      </c>
       <c r="B32">
         <v>31</v>
       </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="C32" s="1">
+        <f t="shared" si="1"/>
+        <v>38.35920177383592</v>
+      </c>
+      <c r="D32">
+        <f t="shared" si="2"/>
+        <v>6.0583333333333336</v>
+      </c>
+      <c r="E32" s="2">
+        <v>45899</v>
+      </c>
+      <c r="F32" s="5">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>10</v>
+      </c>
       <c r="B33">
         <v>32</v>
       </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="C33" s="1">
+        <f t="shared" si="1"/>
+        <v>40.133037694013304</v>
+      </c>
+      <c r="D33">
+        <f t="shared" ref="D33" si="3">AVERAGE(A28:A33)</f>
+        <v>7.3916666666666666</v>
+      </c>
+      <c r="E33" s="2">
+        <v>45900</v>
+      </c>
+      <c r="F33" s="5">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B34">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B35">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B36">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B37">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B38">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B39">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B40">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B41">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B42">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B43">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B44">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B45">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B46">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B47">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B48">
         <v>47</v>
       </c>

</xml_diff>